<commit_message>
add dependency and update it automatically on load (#1159)
</commit_message>
<xml_diff>
--- a/tools/anssi/anssi-guide-hygiene-detail.xlsx
+++ b/tools/anssi/anssi-guide-hygiene-detail.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericlaubacher/Documents/GitHub/ciso-assistant-community/tools/anssi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DC2078-F0B4-3A4A-9947-77E2D878DF09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55C9B573-5E06-0141-879B-B6EA04EC9250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="500" windowWidth="35060" windowHeight="20580" activeTab="1" xr2:uid="{125C4C37-F3C0-444B-A950-381456F8AB10}"/>
+    <workbookView xWindow="780" yWindow="500" windowWidth="35060" windowHeight="20580" xr2:uid="{125C4C37-F3C0-444B-A950-381456F8AB10}"/>
   </bookViews>
   <sheets>
     <sheet name="library_content" sheetId="4" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1208" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="570">
   <si>
     <t>Sensibiliser et former</t>
   </si>
@@ -1899,6 +1899,12 @@
   </si>
   <si>
     <t xml:space="preserve">• les utilisateurs utilisant un poste non administré par le service informatique et qui ne fait pas l’objet de mesures de sécurité édictées par la politique de sécurité générale de l’entité. </t>
+  </si>
+  <si>
+    <t>library_dependencies</t>
+  </si>
+  <si>
+    <t>urn:intuitem:risk:library:doc-pol</t>
   </si>
 </sst>
 </file>
@@ -1977,7 +1983,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2039,9 +2045,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2380,7 +2383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58679FA1-8C3E-D64B-9B35-083A1517BC84}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -2461,45 +2464,42 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>568</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>110</v>
+        <v>569</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>77</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row r="14" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>78</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>79</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -2507,31 +2507,42 @@
         <v>79</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row r="17" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>415</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B17" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="C16">
+      <c r="C17">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B17" s="3"/>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B18" s="1"/>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B19" s="3"/>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B18" s="3"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B19" s="1"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B20" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2640,7 +2651,7 @@
       <c r="C5" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="22" t="s">
         <v>509</v>
       </c>
       <c r="G5" s="4" t="s">
@@ -2660,7 +2671,7 @@
       <c r="C6" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="22" t="s">
         <v>510</v>
       </c>
       <c r="G6" s="4" t="s">
@@ -2680,7 +2691,7 @@
       <c r="C7" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="22" t="s">
         <v>511</v>
       </c>
       <c r="G7" s="4" t="s">
@@ -2700,7 +2711,7 @@
       <c r="C8" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="F8" s="22" t="s">
         <v>512</v>
       </c>
       <c r="G8" s="4" t="s">
@@ -2720,7 +2731,7 @@
       <c r="C9" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="22" t="s">
         <v>513</v>
       </c>
       <c r="G9" s="4" t="s">
@@ -2740,7 +2751,7 @@
       <c r="C10" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="F10" s="22" t="s">
         <v>514</v>
       </c>
       <c r="G10" s="4" t="s">
@@ -2760,7 +2771,7 @@
       <c r="C11" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F11" s="23" t="s">
+      <c r="F11" s="22" t="s">
         <v>515</v>
       </c>
       <c r="G11" s="4" t="s">
@@ -2873,7 +2884,7 @@
       <c r="C17" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F17" s="23" t="s">
+      <c r="F17" s="22" t="s">
         <v>516</v>
       </c>
       <c r="G17" s="4" t="s">
@@ -2893,7 +2904,7 @@
       <c r="C18" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F18" s="23" t="s">
+      <c r="F18" s="22" t="s">
         <v>517</v>
       </c>
       <c r="G18" s="4" t="s">
@@ -2913,7 +2924,7 @@
       <c r="C19" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" s="22" t="s">
         <v>518</v>
       </c>
       <c r="G19" s="4" t="s">
@@ -2933,7 +2944,7 @@
       <c r="C20" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F20" s="23" t="s">
+      <c r="F20" s="22" t="s">
         <v>519</v>
       </c>
       <c r="G20" s="4" t="s">
@@ -2953,7 +2964,7 @@
       <c r="C21" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F21" s="23" t="s">
+      <c r="F21" s="22" t="s">
         <v>520</v>
       </c>
       <c r="G21" s="4" t="s">
@@ -3042,7 +3053,7 @@
       <c r="C26" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F26" s="23" t="s">
+      <c r="F26" s="22" t="s">
         <v>521</v>
       </c>
       <c r="G26" s="4" t="s">
@@ -3062,7 +3073,7 @@
       <c r="C27" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F27" s="23" t="s">
+      <c r="F27" s="22" t="s">
         <v>522</v>
       </c>
       <c r="G27" s="4" t="s">
@@ -3268,7 +3279,7 @@
       <c r="C38" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F38" s="23" t="s">
+      <c r="F38" s="22" t="s">
         <v>523</v>
       </c>
       <c r="G38" s="4" t="s">
@@ -3288,7 +3299,7 @@
       <c r="C39" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F39" s="23" t="s">
+      <c r="F39" s="22" t="s">
         <v>524</v>
       </c>
       <c r="G39" s="4" t="s">
@@ -3308,7 +3319,7 @@
       <c r="C40" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F40" s="23" t="s">
+      <c r="F40" s="22" t="s">
         <v>567</v>
       </c>
       <c r="G40" s="4" t="s">
@@ -3401,7 +3412,7 @@
       <c r="C45" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F45" s="23" t="s">
+      <c r="F45" s="22" t="s">
         <v>525</v>
       </c>
       <c r="G45" s="4" t="s">
@@ -3421,7 +3432,7 @@
       <c r="C46" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F46" s="23" t="s">
+      <c r="F46" s="22" t="s">
         <v>526</v>
       </c>
       <c r="G46" s="4" t="s">
@@ -3441,7 +3452,7 @@
       <c r="C47" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F47" s="23" t="s">
+      <c r="F47" s="22" t="s">
         <v>527</v>
       </c>
       <c r="G47" s="4" t="s">
@@ -3461,7 +3472,7 @@
       <c r="C48" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F48" s="23" t="s">
+      <c r="F48" s="22" t="s">
         <v>528</v>
       </c>
       <c r="G48" s="4" t="s">
@@ -3746,7 +3757,7 @@
       <c r="C63" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F63" s="23" t="s">
+      <c r="F63" s="22" t="s">
         <v>529</v>
       </c>
       <c r="G63" s="4" t="s">
@@ -3766,7 +3777,7 @@
       <c r="C64" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F64" s="23" t="s">
+      <c r="F64" s="22" t="s">
         <v>530</v>
       </c>
       <c r="G64" s="4" t="s">
@@ -3786,7 +3797,7 @@
       <c r="C65" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F65" s="23" t="s">
+      <c r="F65" s="22" t="s">
         <v>531</v>
       </c>
       <c r="G65" s="4" t="s">
@@ -3925,7 +3936,7 @@
       <c r="C72" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F72" s="23" t="s">
+      <c r="F72" s="22" t="s">
         <v>532</v>
       </c>
       <c r="G72" s="4" t="s">
@@ -3945,7 +3956,7 @@
       <c r="C73" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F73" s="23" t="s">
+      <c r="F73" s="22" t="s">
         <v>533</v>
       </c>
       <c r="G73" s="4" t="s">
@@ -3965,7 +3976,7 @@
       <c r="C74" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F74" s="23" t="s">
+      <c r="F74" s="22" t="s">
         <v>534</v>
       </c>
       <c r="G74" s="4" t="s">
@@ -4758,7 +4769,7 @@
       <c r="F114" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="G114" s="22" t="s">
+      <c r="G114" s="4" t="s">
         <v>486</v>
       </c>
       <c r="H114" s="5" t="s">
@@ -4797,7 +4808,7 @@
       <c r="F116" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="G116" s="22" t="s">
+      <c r="G116" s="4" t="s">
         <v>502</v>
       </c>
       <c r="H116" s="4" t="s">
@@ -4820,7 +4831,7 @@
       <c r="F117" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="G117" s="22" t="s">
+      <c r="G117" s="4" t="s">
         <v>487</v>
       </c>
       <c r="I117" s="4" t="s">
@@ -5119,7 +5130,7 @@
       <c r="F132" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="G132" s="22" t="s">
+      <c r="G132" s="4" t="s">
         <v>469</v>
       </c>
       <c r="H132" s="4" t="s">
@@ -5139,7 +5150,7 @@
       <c r="F133" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="G133" s="22" t="s">
+      <c r="G133" s="4" t="s">
         <v>500</v>
       </c>
       <c r="H133" s="4" t="s">
@@ -5162,7 +5173,7 @@
       <c r="F134" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="G134" s="22" t="s">
+      <c r="G134" s="4" t="s">
         <v>501</v>
       </c>
       <c r="H134" s="4" t="s">
@@ -5362,7 +5373,7 @@
       <c r="F144" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="G144" s="22" t="s">
+      <c r="G144" s="4" t="s">
         <v>441</v>
       </c>
       <c r="H144" s="5" t="s">
@@ -5464,7 +5475,7 @@
       <c r="F149" s="4" t="s">
         <v>291</v>
       </c>
-      <c r="G149" s="22" t="s">
+      <c r="G149" s="4" t="s">
         <v>489</v>
       </c>
       <c r="H149" s="5" t="s">
@@ -5687,7 +5698,7 @@
       <c r="F161" s="4" t="s">
         <v>310</v>
       </c>
-      <c r="G161" s="22" t="s">
+      <c r="G161" s="4" t="s">
         <v>507</v>
       </c>
       <c r="H161" s="4" t="s">
@@ -5710,7 +5721,7 @@
       <c r="F162" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="G162" s="22" t="s">
+      <c r="G162" s="4" t="s">
         <v>444</v>
       </c>
       <c r="H162" s="4" t="s">
@@ -5733,7 +5744,7 @@
       <c r="F163" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="G163" s="22" t="s">
+      <c r="G163" s="4" t="s">
         <v>444</v>
       </c>
       <c r="H163" s="4" t="s">
@@ -5756,7 +5767,7 @@
       <c r="F164" s="4" t="s">
         <v>312</v>
       </c>
-      <c r="G164" s="22" t="s">
+      <c r="G164" s="4" t="s">
         <v>444</v>
       </c>
       <c r="H164" s="5" t="s">
@@ -6608,7 +6619,7 @@
       <c r="F210" s="4" t="s">
         <v>549</v>
       </c>
-      <c r="G210" s="22" t="s">
+      <c r="G210" s="4" t="s">
         <v>471</v>
       </c>
       <c r="I210" s="5" t="s">

</xml_diff>

<commit_message>
fix: eager set cast of possibly None implementation_groups field (#1410)
* Fix eager set cast of possibly None implementation_groups field

* fix missing IG

this was causing the issue with null set

---------

Co-authored-by: eric-intuitem <71850047+eric-intuitem@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tools/anssi/anssi-guide-hygiene-detail.xlsx
+++ b/tools/anssi/anssi-guide-hygiene-detail.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericlaubacher/Documents/GitHub/ciso-assistant-community/tools/anssi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A366A31-B445-274E-B43D-59FB50D9B88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC20E2C1-9D63-FD4A-9521-413BDDC1FECA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20580" xr2:uid="{125C4C37-F3C0-444B-A950-381456F8AB10}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="589">
   <si>
     <t>Sensibiliser et former</t>
   </si>
@@ -2074,6 +2074,9 @@
 Vérifier que le référent est responsable de la vérification de l’application des règles.
 Vérifier que le référent est responsable de la sensibilisation des utilisateurs et de la définition d’un plan de formation des acteurs informatiques.
 Vérifier que le référent est responsable de la centralisation et du traitement des incidents de sécurité constatés ou remontés par les utilisateurs.</t>
+  </si>
+  <si>
+    <t>library_publication_date</t>
   </si>
 </sst>
 </file>
@@ -2139,7 +2142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2198,6 +2201,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2533,7 +2539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58679FA1-8C3E-D64B-9B35-083A1517BC84}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -2553,7 +2559,7 @@
         <v>66</v>
       </c>
       <c r="B2" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -2566,101 +2572,98 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>112</v>
+        <v>588</v>
+      </c>
+      <c r="B4" s="21">
+        <v>45680</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="7" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>71</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>407</v>
+        <v>73</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>408</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>407</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>110</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>77</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="51" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+    <row r="15" spans="1:3" ht="51" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>78</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B15" s="3" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C15" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -2668,31 +2671,42 @@
         <v>79</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C17" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="18" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>257</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="C17">
+      <c r="C18">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="3"/>
-    </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B19" s="1"/>
+      <c r="B19" s="3"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B20" s="3"/>
+      <c r="B20" s="1"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3499,6 +3513,9 @@
       <c r="B44" s="4">
         <v>3</v>
       </c>
+      <c r="C44" s="4" t="s">
+        <v>85</v>
+      </c>
       <c r="F44" s="4" t="s">
         <v>133</v>
       </c>

</xml_diff>